<commit_message>
Add IndusInd Bank and IDFC FIRST Bank custom parsers
- Implemented custom parser for IndusInd Bank (14 rates extracted)
  * Extracts annualized yield columns for deposits < 3 Cr
  * Columns: Annualized Yield (General) and (Senior Citizen)

- Implemented custom parser for IDFC FIRST Bank (13 rates extracted)
  * Standard table parser for deposits < ₹3 Crore
  * Extracts general and senior citizen rates

- Updated extraction results: 209 total rates from 18 banks (60% success)
- Added comprehensive final extraction report
- Updated bank URLs in Excel file
- Added test scripts for both new parsers

Total custom parsers: 15 (including 2 new parsers)
</commit_message>
<xml_diff>
--- a/List_of_Banksv1.xlsx
+++ b/List_of_Banksv1.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Shared/Shared-d/Famli/Prototype/Bank FD Rates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3BC0728-ED6F-8D45-88BF-BF6709862070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A4A2B94-6913-DF44-8931-5555145E1D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="184">
   <si>
     <t>bank_id</t>
   </si>
@@ -184,9 +197,6 @@
     <t>https://www.axisbank.com</t>
   </si>
   <si>
-    <t>https://www.axisbank.com/business-banking/interest-rates-and-derivatives</t>
-  </si>
-  <si>
     <t>KOTAK</t>
   </si>
   <si>
@@ -205,9 +215,6 @@
     <t>https://www.indusind.com</t>
   </si>
   <si>
-    <t>https://www.indusind.bank.in/in/en/personal/deposits/fixed-deposit.html</t>
-  </si>
-  <si>
     <t>YES</t>
   </si>
   <si>
@@ -238,9 +245,6 @@
     <t>https://www.idfcfirstbank.com</t>
   </si>
   <si>
-    <t>https://www.idfcfirstbank.com/nri-banking/nri-fixed-deposit</t>
-  </si>
-  <si>
     <t>FEDERAL</t>
   </si>
   <si>
@@ -563,6 +567,24 @@
   </si>
   <si>
     <t>https://pnb.bank.in/Interest-Rates-Deposit.html</t>
+  </si>
+  <si>
+    <t>https://bankofbaroda.bank.in/interest-rate-and-service-charges/deposits-interest-rates/fixed-deposits-callable-and-non-callable-upto-ten-crores</t>
+  </si>
+  <si>
+    <t>https://www.axis.bank.in/docs/default-source/default-document-library/interest-rates/domestic-fixed-deposits-05-may-26.pdf</t>
+  </si>
+  <si>
+    <t>https://www.au.bank.in/interest-rates/fixed-deposit-interest-rates</t>
+  </si>
+  <si>
+    <t>https://www.unionbankofindia.bank.in/en/details/rate-of-interest</t>
+  </si>
+  <si>
+    <t>https://www.indusind.bank.in/in/en/personal/fixed-deposit-interest-rate.html</t>
+  </si>
+  <si>
+    <t>https://www.idfcfirst.bank.in/personal-banking/deposits/fixed-deposit/fd-interest-rates</t>
   </si>
 </sst>
 </file>
@@ -988,10 +1010,10 @@
         <v>10</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -1014,7 +1036,7 @@
         <v>14</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -1037,7 +1059,7 @@
         <v>18</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -1057,10 +1079,10 @@
         <v>21</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -1082,6 +1104,9 @@
       <c r="F6" s="2" t="s">
         <v>24</v>
       </c>
+      <c r="G6" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
@@ -1100,7 +1125,10 @@
         <v>10</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
+      </c>
+      <c r="G7" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -1120,7 +1148,7 @@
         <v>29</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -1140,10 +1168,10 @@
         <v>10</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -1163,10 +1191,10 @@
         <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1186,10 +1214,10 @@
         <v>36</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="G11" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -1232,7 +1260,7 @@
         <v>43</v>
       </c>
       <c r="G13" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1255,7 +1283,7 @@
         <v>47</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -1278,7 +1306,7 @@
         <v>50</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1301,7 +1329,7 @@
         <v>53</v>
       </c>
       <c r="G16" t="s">
-        <v>54</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1309,10 +1337,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" t="s">
         <v>55</v>
-      </c>
-      <c r="C17" t="s">
-        <v>56</v>
       </c>
       <c r="D17" t="s">
         <v>46</v>
@@ -1321,10 +1349,10 @@
         <v>10</v>
       </c>
       <c r="F17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G17" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1332,10 +1360,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" t="s">
         <v>58</v>
-      </c>
-      <c r="C18" t="s">
-        <v>59</v>
       </c>
       <c r="D18" t="s">
         <v>46</v>
@@ -1344,10 +1372,10 @@
         <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G18" t="s">
-        <v>61</v>
+        <v>182</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1355,10 +1383,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
         <v>46</v>
@@ -1367,10 +1395,10 @@
         <v>10</v>
       </c>
       <c r="F19" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G19" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1378,10 +1406,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C20" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
         <v>46</v>
@@ -1390,10 +1418,10 @@
         <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G20" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1401,10 +1429,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D21" t="s">
         <v>46</v>
@@ -1413,10 +1441,10 @@
         <v>10</v>
       </c>
       <c r="F21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G21" t="s">
-        <v>72</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1424,22 +1452,22 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C22" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D22" t="s">
         <v>46</v>
       </c>
       <c r="E22" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="G22" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1447,19 +1475,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C23" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D23" t="s">
         <v>46</v>
       </c>
       <c r="E23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1467,10 +1495,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C24" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D24" t="s">
         <v>46</v>
@@ -1479,10 +1507,10 @@
         <v>36</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G24" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1490,10 +1518,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D25" t="s">
         <v>46</v>
@@ -1502,10 +1530,10 @@
         <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G25" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1513,22 +1541,22 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C26" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D26" t="s">
         <v>46</v>
       </c>
       <c r="E26" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F26" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G26" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1536,22 +1564,22 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C27" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D27" t="s">
         <v>46</v>
       </c>
       <c r="E27" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F27" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G27" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1559,22 +1587,22 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C28" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D28" t="s">
         <v>46</v>
       </c>
       <c r="E28" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F28" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G28" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1582,19 +1610,22 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
+        <v>100</v>
+      </c>
+      <c r="C29" t="s">
+        <v>101</v>
+      </c>
+      <c r="D29" t="s">
+        <v>102</v>
+      </c>
+      <c r="E29" t="s">
         <v>103</v>
       </c>
-      <c r="C29" t="s">
+      <c r="F29" t="s">
         <v>104</v>
       </c>
-      <c r="D29" t="s">
-        <v>105</v>
-      </c>
-      <c r="E29" t="s">
-        <v>106</v>
-      </c>
-      <c r="F29" t="s">
-        <v>107</v>
+      <c r="G29" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -1602,19 +1633,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C30" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D30" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E30" t="s">
         <v>29</v>
       </c>
       <c r="F30" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1622,22 +1653,22 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C31" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D31" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E31" t="s">
         <v>21</v>
       </c>
       <c r="F31" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G31" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1645,22 +1676,22 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
+        <v>112</v>
+      </c>
+      <c r="C32" t="s">
+        <v>113</v>
+      </c>
+      <c r="D32" t="s">
+        <v>102</v>
+      </c>
+      <c r="E32" t="s">
+        <v>114</v>
+      </c>
+      <c r="F32" t="s">
         <v>115</v>
       </c>
-      <c r="C32" t="s">
+      <c r="G32" t="s">
         <v>116</v>
-      </c>
-      <c r="D32" t="s">
-        <v>105</v>
-      </c>
-      <c r="E32" t="s">
-        <v>117</v>
-      </c>
-      <c r="F32" t="s">
-        <v>118</v>
-      </c>
-      <c r="G32" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1668,19 +1699,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C33" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D33" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E33" t="s">
         <v>21</v>
       </c>
       <c r="F33" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1688,19 +1719,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C34" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D34" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E34" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F34" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1708,22 +1739,22 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
+        <v>123</v>
+      </c>
+      <c r="C35" t="s">
+        <v>124</v>
+      </c>
+      <c r="D35" t="s">
+        <v>102</v>
+      </c>
+      <c r="E35" t="s">
+        <v>125</v>
+      </c>
+      <c r="F35" t="s">
         <v>126</v>
       </c>
-      <c r="C35" t="s">
+      <c r="G35" t="s">
         <v>127</v>
-      </c>
-      <c r="D35" t="s">
-        <v>105</v>
-      </c>
-      <c r="E35" t="s">
-        <v>128</v>
-      </c>
-      <c r="F35" t="s">
-        <v>129</v>
-      </c>
-      <c r="G35" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1731,19 +1762,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
+        <v>128</v>
+      </c>
+      <c r="C36" t="s">
+        <v>129</v>
+      </c>
+      <c r="D36" t="s">
+        <v>102</v>
+      </c>
+      <c r="E36" t="s">
+        <v>130</v>
+      </c>
+      <c r="F36" t="s">
         <v>131</v>
-      </c>
-      <c r="C36" t="s">
-        <v>132</v>
-      </c>
-      <c r="D36" t="s">
-        <v>105</v>
-      </c>
-      <c r="E36" t="s">
-        <v>133</v>
-      </c>
-      <c r="F36" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1751,22 +1782,22 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C37" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D37" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E37" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F37" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="G37" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1774,22 +1805,22 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C38" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D38" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
       </c>
       <c r="F38" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G38" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1797,19 +1828,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C39" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D39" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E39" t="s">
         <v>13</v>
       </c>
       <c r="F39" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1817,19 +1848,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C40" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D40" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E40" t="s">
         <v>13</v>
       </c>
       <c r="F40" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1837,19 +1868,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C41" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D41" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E41" t="s">
         <v>10</v>
       </c>
       <c r="F41" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1857,19 +1888,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C42" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D42" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E42" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F42" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1877,37 +1908,36 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C43" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D43" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="E43" t="s">
         <v>10</v>
       </c>
       <c r="F43" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="G15" r:id="rId1" xr:uid="{1509A87A-1F98-4CFA-82E2-D91DBB065CA5}"/>
     <hyperlink ref="F2" r:id="rId2" xr:uid="{58507B79-4185-F947-A4AB-98C9919B29B2}"/>
-    <hyperlink ref="G4" r:id="rId3" xr:uid="{9F79BB46-25D4-804E-AFC8-AC46FEC95842}"/>
-    <hyperlink ref="F5" r:id="rId4" xr:uid="{BAA03276-CDA2-4042-8DD6-CC492424C534}"/>
-    <hyperlink ref="G5" r:id="rId5" xr:uid="{C2B519E0-C065-644A-A428-BCF0E58C5BE2}"/>
-    <hyperlink ref="F6" r:id="rId6" xr:uid="{CEA22EB3-16AB-084A-930A-C8D68B903965}"/>
-    <hyperlink ref="F7" r:id="rId7" xr:uid="{972BE229-7971-F641-8EF8-B805FD92B0BC}"/>
-    <hyperlink ref="F8" r:id="rId8" xr:uid="{AEAB195E-52B3-7045-9E5A-0F2EB1C35F22}"/>
-    <hyperlink ref="F9" r:id="rId9" xr:uid="{080E18B2-3A18-ED40-B23A-CE9644955768}"/>
-    <hyperlink ref="G9" r:id="rId10" xr:uid="{A0CCD28D-A625-204C-ADAF-03137F45877F}"/>
-    <hyperlink ref="G10" r:id="rId11" xr:uid="{6AB966F3-BC23-E549-B47F-05E98F791A04}"/>
-    <hyperlink ref="F11" r:id="rId12" xr:uid="{509CB66E-AA3F-6746-A754-92C67E96885E}"/>
-    <hyperlink ref="G14" r:id="rId13" xr:uid="{CBDA1605-68A4-E44B-8C87-52154F102C02}"/>
-    <hyperlink ref="G2" r:id="rId14" xr:uid="{294B4D14-7891-E345-9EE4-39D77A6BAB6F}"/>
+    <hyperlink ref="F5" r:id="rId3" xr:uid="{BAA03276-CDA2-4042-8DD6-CC492424C534}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{C2B519E0-C065-644A-A428-BCF0E58C5BE2}"/>
+    <hyperlink ref="F6" r:id="rId5" xr:uid="{CEA22EB3-16AB-084A-930A-C8D68B903965}"/>
+    <hyperlink ref="F7" r:id="rId6" xr:uid="{972BE229-7971-F641-8EF8-B805FD92B0BC}"/>
+    <hyperlink ref="F8" r:id="rId7" xr:uid="{AEAB195E-52B3-7045-9E5A-0F2EB1C35F22}"/>
+    <hyperlink ref="F9" r:id="rId8" xr:uid="{080E18B2-3A18-ED40-B23A-CE9644955768}"/>
+    <hyperlink ref="G9" r:id="rId9" xr:uid="{A0CCD28D-A625-204C-ADAF-03137F45877F}"/>
+    <hyperlink ref="G10" r:id="rId10" xr:uid="{6AB966F3-BC23-E549-B47F-05E98F791A04}"/>
+    <hyperlink ref="F11" r:id="rId11" xr:uid="{509CB66E-AA3F-6746-A754-92C67E96885E}"/>
+    <hyperlink ref="G14" r:id="rId12" xr:uid="{CBDA1605-68A4-E44B-8C87-52154F102C02}"/>
+    <hyperlink ref="G2" r:id="rId13" xr:uid="{294B4D14-7891-E345-9EE4-39D77A6BAB6F}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>